<commit_message>
core measurement record updated
</commit_message>
<xml_diff>
--- a/notes/coreMeasurement/coresScanned.xlsx
+++ b/notes/coreMeasurement/coresScanned.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PhD\Project\PhD_thesis\mast_growth\notes\coreMeasurement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D75C2AEA-5A8D-41E8-8B63-843F97D96015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF23D0D7-1011-4D78-8D0B-55B428141AFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="760" windowWidth="14400" windowHeight="7350" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="380" yWindow="380" windowWidth="14400" windowHeight="7350" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AB08" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4041" uniqueCount="1257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4043" uniqueCount="1257">
   <si>
     <t>Stand</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -11663,6 +11663,18 @@
       <c r="C27" s="2" t="s">
         <v>232</v>
       </c>
+      <c r="D27" s="2" t="s">
+        <v>1246</v>
+      </c>
+      <c r="E27" s="6">
+        <v>46272</v>
+      </c>
+      <c r="F27">
+        <v>130</v>
+      </c>
+      <c r="G27">
+        <v>0.87</v>
+      </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
@@ -11673,6 +11685,18 @@
       </c>
       <c r="C28" s="2" t="s">
         <v>232</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>1246</v>
+      </c>
+      <c r="E28" s="6">
+        <v>46272</v>
+      </c>
+      <c r="F28">
+        <v>130</v>
+      </c>
+      <c r="G28">
+        <v>0.87</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
core measurement record updates
</commit_message>
<xml_diff>
--- a/notes/coreMeasurement/coresScanned.xlsx
+++ b/notes/coreMeasurement/coresScanned.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PhD\Project\PhD_thesis\mast_growth\notes\coreMeasurement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF23D0D7-1011-4D78-8D0B-55B428141AFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78860D23-10BC-4294-A223-AF3900F95F3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="380" windowWidth="14400" windowHeight="7350" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AB08" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4043" uniqueCount="1257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4044" uniqueCount="1257">
   <si>
     <t>Stand</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -11709,6 +11709,15 @@
       <c r="C29" s="2" t="s">
         <v>232</v>
       </c>
+      <c r="D29" s="2" t="s">
+        <v>1246</v>
+      </c>
+      <c r="E29" s="6">
+        <v>46275</v>
+      </c>
+      <c r="F29">
+        <v>130</v>
+      </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">

</xml_diff>

<commit_message>
edits the core measurement sheet format
</commit_message>
<xml_diff>
--- a/notes/coreMeasurement/coresScanned.xlsx
+++ b/notes/coreMeasurement/coresScanned.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PhD\Project\PhD_thesis\mast_growth\notes\coreMeasurement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78860D23-10BC-4294-A223-AF3900F95F3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D704CA7-3959-4C7A-8D90-80D24A90EFDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4044" uniqueCount="1257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4045" uniqueCount="1257">
   <si>
     <t>Stand</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -11729,6 +11729,18 @@
       <c r="C30" s="2" t="s">
         <v>232</v>
       </c>
+      <c r="D30" s="2" t="s">
+        <v>1246</v>
+      </c>
+      <c r="E30" s="6">
+        <v>46280</v>
+      </c>
+      <c r="F30">
+        <v>130</v>
+      </c>
+      <c r="G30">
+        <v>0.73</v>
+      </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">

</xml_diff>